<commit_message>
Update SP0557_rev02 AI3_2 Excel file
Replace the binary Excel (.xlsx) file under PCBNo.10081/SP0557_rev02_00_AI3/SP0557_rev02_00_AI3_2. The spreadsheet contents were changed (binary diff), likely updating BOM/assembly data or revision details for SP0557 rev02; no textual diff available.
</commit_message>
<xml_diff>
--- a/PCBNo.10081/PCBNo.10081/SP0557_rev02_00_AI3/SP0557_rev02_00_AI3_2/修正履歴.xlsx
+++ b/PCBNo.10081/PCBNo.10081/SP0557_rev02_00_AI3/SP0557_rev02_00_AI3_2/修正履歴.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\work\S127M\PCBNo_10081\SP0557_rev02_00_AI3\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/512e22ffcc52695f/ドキュメント/GitHub/PCBNo.10081/PCBNo.10081/PCBNo.10081/SP0557_rev02_00_AI3/SP0557_rev02_00_AI3_2/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BCDA7BAB-8026-4C53-BAA1-6CFCABC79B71}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="17" documentId="13_ncr:1_{BCDA7BAB-8026-4C53-BAA1-6CFCABC79B71}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{41E34AB5-8F88-49EF-A593-73BDE1461DFE}"/>
   <bookViews>
-    <workbookView xWindow="-80" yWindow="-80" windowWidth="21760" windowHeight="13840" activeTab="6" xr2:uid="{3A2BB469-6CC5-41C3-8C98-63503D4CF60C}"/>
+    <workbookView xWindow="-16320" yWindow="-120" windowWidth="16440" windowHeight="28320" firstSheet="1" activeTab="7" xr2:uid="{3A2BB469-6CC5-41C3-8C98-63503D4CF60C}"/>
   </bookViews>
   <sheets>
     <sheet name="修正履歴" sheetId="1" r:id="rId1"/>
@@ -20,6 +20,7 @@
     <sheet name="No4" sheetId="5" r:id="rId5"/>
     <sheet name="No5" sheetId="7" r:id="rId6"/>
     <sheet name="No6" sheetId="8" r:id="rId7"/>
+    <sheet name="No.7" sheetId="9" r:id="rId8"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -42,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="768" uniqueCount="676">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="806" uniqueCount="710">
   <si>
     <t>No</t>
     <phoneticPr fontId="1"/>
@@ -4899,12 +4900,245 @@
     <t>4. Synplify で再合成 → automake.log で以下を確認:</t>
     <phoneticPr fontId="1"/>
   </si>
+  <si>
+    <t>７</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>No6で解消しなかったため、追加解析</t>
+    <rPh sb="4" eb="6">
+      <t>カイショウ</t>
+    </rPh>
+    <rPh sb="14" eb="16">
+      <t>ツイカ</t>
+    </rPh>
+    <rPh sb="16" eb="18">
+      <t>カイセキ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>No.6 実装の問題点と今回の対策</t>
+  </si>
+  <si>
+    <t>問題の核心</t>
+  </si>
+  <si>
+    <t>問題点（3つ）</t>
+  </si>
+  <si>
+    <t>1. FDCのクロックネット名が間違っていた</t>
+  </si>
+  <si>
+    <t>FDCでPLL出力クロックを定義する際、pll_gen内に存在しない信号名を参照していました。</t>
+  </si>
+  <si>
+    <t>誤: {n:slv_com_top_inst.clk_gen_inst2.PLL_inst.CLKCOM_OUT}  ← pll_gen内に存在しない</t>
+  </si>
+  <si>
+    <t>正: {p:CLKOP}                                                ← pll_genの実際のポート名</t>
+  </si>
+  <si>
+    <t>2. AutoConstraint_SP0557.sdc が無効化されていなかった</t>
+  </si>
+  <si>
+    <t>.sdc.bak にリネームしたつもりが、元の .sdc も残っており、Synplifyがこの間違った制約を読み込んでいました。内容は：</t>
+  </si>
+  <si>
+    <t>この設定により、SDCファイルを削除しても合成のたびにSynplifyが同じ間違った内容で再生成します。</t>
+  </si>
+  <si>
+    <t>結果として起きていたこと</t>
+  </si>
+  <si>
+    <t>今回の対策（5ファイル修正）</t>
+  </si>
+  <si>
+    <t>対策</t>
+  </si>
+  <si>
+    <t>内容</t>
+  </si>
+  <si>
+    <t>FDCネット名修正</t>
+  </si>
+  <si>
+    <t>pll_gen.fdc</t>
+  </si>
+  <si>
+    <t>FDC役割分離</t>
+  </si>
+  <si>
+    <t>クロック定義を削除し、マルチサイクル/フォールスパス制約のみに変更</t>
+  </si>
+  <si>
+    <t>SDC無効化</t>
+  </si>
+  <si>
+    <t>間違った制約を全削除</t>
+  </si>
+  <si>
+    <t>自動再生成防止</t>
+  </si>
+  <si>
+    <t>SP0557_syn.prj</t>
+  </si>
+  <si>
+    <t>LPFネット名修正</t>
+  </si>
+  <si>
+    <r>
+      <t>No.6で追加したタイミング制約が</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Meiryo UI"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>全てSynplifyに無視されていた</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Meiryo UI"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>ため、エラーが解消しませんでした。</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>CLKCOM_OUT, CLK2A, s_PLL_CLK20M, CLK1 はいずれもslv_com_top.vhdの信号名であり、pll_gen内部のポート名（CLKOP, CLKOS, CLKOS2, CLKOS3）とは一致しません。Synplifyはマッチしない制約をサイレントに無視するため、</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Meiryo UI"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>同一クロックグループ設定が一切適用されていませんでした</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Meiryo UI"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>。</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>全PLLクロックが</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Meiryo UI"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>別々のクロックグループ</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Meiryo UI"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>（Autoconstr_clkgroup_0〜4）</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>間違った周期</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Meiryo UI"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>（20MHzが6.2ns=161MHz、100MHzが3.5ns=286MHz等）</t>
+    </r>
+  </si>
+  <si>
+    <t>3. set_option -frequency auto が自動再生成を引き起こす</t>
+  </si>
+  <si>
+    <r>
+      <t>CLK2（100MHz, 0°）とCLK2A（100MHz, 90°）が</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Meiryo UI"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>別クロックグループ</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Meiryo UI"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>に分類され、cds.vhd（CDRモジュール）のクロスドメインパスが</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Meiryo UI"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>完全に未タイミング解析</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Meiryo UI"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>。LE占有率80%でルーティングが混雑した際にこれらのパスがタイミング違反を起こし、通信エラーが発生。</t>
+    </r>
+  </si>
+  <si>
+    <t>PLLモジュール内で{p:CLKOP}等のポート参照を使用。全クロックを同一グループpll_clksに配置</t>
+  </si>
+  <si>
+    <t>frequency auto→100.0、pll_gen.fdc を明示的に追加</t>
+  </si>
+  <si>
+    <t>CLKCOM_OUT→CLK2（open接続のため不存在）、/CLK2A→.CLK2A（区切り文字統一）</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="25">
+  <fonts count="27">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -5085,6 +5319,20 @@
       <family val="3"/>
       <charset val="128"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Meiryo UI"/>
+      <family val="3"/>
+      <charset val="128"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Meiryo UI"/>
+      <family val="3"/>
+      <charset val="128"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -5150,7 +5398,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="72">
+  <cellXfs count="82">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -5366,6 +5614,36 @@
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -5702,11 +5980,11 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8D0ED093-D5BA-4371-A312-AC8F17AA5EBD}">
   <dimension ref="C4:F32"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15.75"/>
   <cols>
     <col min="1" max="3" width="9" style="28"/>
     <col min="4" max="4" width="9.25" style="28" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="48.58203125" style="28" customWidth="1"/>
+    <col min="5" max="5" width="48.625" style="28" customWidth="1"/>
     <col min="6" max="6" width="43.5" style="28" customWidth="1"/>
     <col min="7" max="16384" width="9" style="28"/>
   </cols>
@@ -5802,9 +6080,15 @@
       <c r="F10" s="26"/>
     </row>
     <row r="11" spans="3:6">
-      <c r="C11" s="26"/>
-      <c r="D11" s="29"/>
-      <c r="E11" s="27"/>
+      <c r="C11" s="26">
+        <v>7</v>
+      </c>
+      <c r="D11" s="29" t="s">
+        <v>676</v>
+      </c>
+      <c r="E11" s="27" t="s">
+        <v>677</v>
+      </c>
       <c r="F11" s="26"/>
     </row>
     <row r="12" spans="3:6">
@@ -5942,21 +6226,21 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3F89F06B-6716-43FB-A17C-800E0158B134}">
   <dimension ref="B2:D43"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15.75"/>
   <cols>
     <col min="1" max="1" width="9" style="1"/>
-    <col min="2" max="2" width="84.33203125" style="1" customWidth="1"/>
+    <col min="2" max="2" width="84.375" style="1" customWidth="1"/>
     <col min="3" max="3" width="35.5" style="1" customWidth="1"/>
-    <col min="4" max="4" width="35.58203125" style="1" customWidth="1"/>
+    <col min="4" max="4" width="35.625" style="1" customWidth="1"/>
     <col min="5" max="16384" width="9" style="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:4" ht="24.5">
+    <row r="2" spans="2:4" ht="24">
       <c r="B2" s="2" t="s">
         <v>130</v>
       </c>
     </row>
-    <row r="3" spans="2:4" ht="19">
+    <row r="3" spans="2:4" ht="18.75">
       <c r="B3" s="3" t="s">
         <v>131</v>
       </c>
@@ -5972,7 +6256,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="5" spans="2:4" ht="15.5" thickBot="1">
+    <row r="5" spans="2:4" ht="16.5" thickBot="1">
       <c r="B5" s="6" t="s">
         <v>166</v>
       </c>
@@ -5983,7 +6267,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="6" spans="2:4" ht="15.5" thickBot="1">
+    <row r="6" spans="2:4" ht="16.5" thickBot="1">
       <c r="B6" s="6" t="s">
         <v>167</v>
       </c>
@@ -5994,7 +6278,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="7" spans="2:4" ht="15.5" thickBot="1">
+    <row r="7" spans="2:4" ht="16.5" thickBot="1">
       <c r="B7" s="6" t="s">
         <v>139</v>
       </c>
@@ -6016,7 +6300,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="9" spans="2:4" ht="19">
+    <row r="9" spans="2:4" ht="18.75">
       <c r="B9" s="3" t="s">
         <v>145</v>
       </c>
@@ -6078,7 +6362,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="27" spans="2:2" ht="19">
+    <row r="27" spans="2:2" ht="18.75">
       <c r="B27" s="3" t="s">
         <v>154</v>
       </c>
@@ -6101,7 +6385,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="33" spans="2:4" ht="19">
+    <row r="33" spans="2:4" ht="18.75">
       <c r="B33" s="3" t="s">
         <v>156</v>
       </c>
@@ -6117,7 +6401,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="35" spans="2:4" ht="15.5" thickBot="1">
+    <row r="35" spans="2:4" ht="16.5" thickBot="1">
       <c r="B35" s="7" t="s">
         <v>117</v>
       </c>
@@ -6128,7 +6412,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="36" spans="2:4" ht="15.5" thickBot="1">
+    <row r="36" spans="2:4" ht="16.5" thickBot="1">
       <c r="B36" s="7" t="s">
         <v>158</v>
       </c>
@@ -6150,7 +6434,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="38" spans="2:4" ht="19">
+    <row r="38" spans="2:4" ht="18.75">
       <c r="B38" s="3" t="s">
         <v>163</v>
       </c>
@@ -6187,16 +6471,16 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B32F4D81-2017-4BFB-925A-9B9391062D61}">
   <dimension ref="B2:D139"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15.75"/>
   <cols>
     <col min="1" max="1" width="9" style="1"/>
-    <col min="2" max="2" width="20.33203125" style="1" customWidth="1"/>
-    <col min="3" max="3" width="57.58203125" style="1" customWidth="1"/>
-    <col min="4" max="4" width="44.58203125" style="1" customWidth="1"/>
+    <col min="2" max="2" width="20.375" style="1" customWidth="1"/>
+    <col min="3" max="3" width="57.625" style="1" customWidth="1"/>
+    <col min="4" max="4" width="44.625" style="1" customWidth="1"/>
     <col min="5" max="16384" width="9" style="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:2" ht="24.5">
+    <row r="2" spans="2:2" ht="24">
       <c r="B2" s="14" t="s">
         <v>9</v>
       </c>
@@ -6206,7 +6490,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="6" spans="2:2" ht="19">
+    <row r="6" spans="2:2" ht="18.75">
       <c r="B6" s="15" t="s">
         <v>10</v>
       </c>
@@ -6284,12 +6568,12 @@
         <v>22</v>
       </c>
     </row>
-    <row r="29" spans="2:2" ht="24.5">
+    <row r="29" spans="2:2" ht="24">
       <c r="B29" s="14" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="31" spans="2:2" ht="19">
+    <row r="31" spans="2:2" ht="18.75">
       <c r="B31" s="15" t="s">
         <v>24</v>
       </c>
@@ -6397,7 +6681,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="58" spans="2:2" ht="19">
+    <row r="58" spans="2:2" ht="18.75">
       <c r="B58" s="15" t="s">
         <v>41</v>
       </c>
@@ -6437,7 +6721,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="68" spans="2:2" ht="19">
+    <row r="68" spans="2:2" ht="18.75">
       <c r="B68" s="15" t="s">
         <v>47</v>
       </c>
@@ -6477,7 +6761,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="78" spans="2:2" ht="19">
+    <row r="78" spans="2:2" ht="18.75">
       <c r="B78" s="15" t="s">
         <v>53</v>
       </c>
@@ -6530,7 +6814,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="95" spans="2:2" ht="24.5">
+    <row r="95" spans="2:2" ht="24">
       <c r="B95" s="14" t="s">
         <v>62</v>
       </c>
@@ -6557,7 +6841,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="101" spans="2:4" ht="24.5">
+    <row r="101" spans="2:4" ht="24">
       <c r="B101" s="14" t="s">
         <v>69</v>
       </c>
@@ -6639,7 +6923,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="111" spans="2:4" ht="24.5">
+    <row r="111" spans="2:4" ht="24">
       <c r="B111" s="14" t="s">
         <v>88</v>
       </c>
@@ -6666,7 +6950,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="115" spans="2:4" ht="30">
+    <row r="115" spans="2:4" ht="31.5">
       <c r="B115" s="9" t="s">
         <v>95</v>
       </c>
@@ -6677,7 +6961,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="116" spans="2:4" ht="30">
+    <row r="116" spans="2:4" ht="31.5">
       <c r="B116" s="9" t="s">
         <v>98</v>
       </c>
@@ -6688,7 +6972,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="117" spans="2:4" ht="30">
+    <row r="117" spans="2:4" ht="31.5">
       <c r="B117" s="9" t="s">
         <v>101</v>
       </c>
@@ -6699,7 +6983,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="120" spans="2:4" ht="24.5">
+    <row r="120" spans="2:4" ht="24">
       <c r="B120" s="14" t="s">
         <v>104</v>
       </c>
@@ -6715,7 +6999,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="123" spans="2:4" ht="30">
+    <row r="123" spans="2:4" ht="31.5">
       <c r="B123" s="9" t="s">
         <v>108</v>
       </c>
@@ -6726,7 +7010,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="124" spans="2:4" ht="30">
+    <row r="124" spans="2:4" ht="31.5">
       <c r="B124" s="9" t="s">
         <v>111</v>
       </c>
@@ -6770,7 +7054,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="130" spans="2:2" ht="24.5">
+    <row r="130" spans="2:2" ht="24">
       <c r="B130" s="14" t="s">
         <v>122</v>
       </c>
@@ -6827,10 +7111,10 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5E81A2F4-F9B4-404A-AE58-E34E7E0FCE12}">
   <dimension ref="B2:B171"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15.75"/>
   <cols>
     <col min="1" max="1" width="9" style="1"/>
-    <col min="2" max="2" width="255.58203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="255.625" style="1" bestFit="1" customWidth="1"/>
     <col min="3" max="16384" width="9" style="1"/>
   </cols>
   <sheetData>
@@ -7453,11 +7737,11 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A08E866B-9F97-45D7-AE69-ACECA99C7B6F}">
   <dimension ref="B2:E92"/>
-  <sheetFormatPr defaultRowHeight="18"/>
+  <sheetFormatPr defaultRowHeight="18.75"/>
   <cols>
     <col min="2" max="2" width="40.5" customWidth="1"/>
-    <col min="3" max="3" width="39.08203125" customWidth="1"/>
-    <col min="4" max="4" width="79.33203125" customWidth="1"/>
+    <col min="3" max="3" width="39.125" customWidth="1"/>
+    <col min="4" max="4" width="79.375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="2:2">
@@ -7466,7 +7750,7 @@
     <row r="3" spans="2:2">
       <c r="B3" s="35"/>
     </row>
-    <row r="4" spans="2:2" ht="29">
+    <row r="4" spans="2:2" ht="30">
       <c r="B4" s="41" t="s">
         <v>465</v>
       </c>
@@ -7485,7 +7769,7 @@
     <row r="9" spans="2:2">
       <c r="B9" s="35"/>
     </row>
-    <row r="10" spans="2:2" ht="29">
+    <row r="10" spans="2:2" ht="30">
       <c r="B10" s="41" t="s">
         <v>467</v>
       </c>
@@ -7493,7 +7777,7 @@
     <row r="11" spans="2:2">
       <c r="B11" s="35"/>
     </row>
-    <row r="12" spans="2:2" ht="22">
+    <row r="12" spans="2:2" ht="22.5">
       <c r="B12" s="42" t="s">
         <v>468</v>
       </c>
@@ -7545,7 +7829,7 @@
         <v>478</v>
       </c>
     </row>
-    <row r="20" spans="2:5" ht="36">
+    <row r="20" spans="2:5" ht="36.75">
       <c r="B20" s="43" t="s">
         <v>479</v>
       </c>
@@ -7612,7 +7896,7 @@
     <row r="26" spans="2:5">
       <c r="B26" s="35"/>
     </row>
-    <row r="27" spans="2:5" ht="22">
+    <row r="27" spans="2:5" ht="22.5">
       <c r="B27" s="42" t="s">
         <v>493</v>
       </c>
@@ -7636,7 +7920,7 @@
         <v>496</v>
       </c>
     </row>
-    <row r="32" spans="2:5" ht="36">
+    <row r="32" spans="2:5" ht="37.5">
       <c r="B32" s="32" t="s">
         <v>497</v>
       </c>
@@ -7644,7 +7928,7 @@
         <v>498</v>
       </c>
     </row>
-    <row r="33" spans="2:4" ht="36">
+    <row r="33" spans="2:4" ht="37.5">
       <c r="B33" s="32" t="s">
         <v>499</v>
       </c>
@@ -7652,7 +7936,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="34" spans="2:4" ht="36">
+    <row r="34" spans="2:4" ht="37.5">
       <c r="B34" s="32" t="s">
         <v>501</v>
       </c>
@@ -7671,7 +7955,7 @@
     <row r="37" spans="2:4">
       <c r="B37" s="35"/>
     </row>
-    <row r="38" spans="2:4" ht="22">
+    <row r="38" spans="2:4" ht="22.5">
       <c r="B38" s="42" t="s">
         <v>504</v>
       </c>
@@ -7745,7 +8029,7 @@
     <row r="50" spans="2:5">
       <c r="B50" s="35"/>
     </row>
-    <row r="51" spans="2:5" ht="29">
+    <row r="51" spans="2:5" ht="30">
       <c r="B51" s="41" t="s">
         <v>514</v>
       </c>
@@ -7837,7 +8121,7 @@
     <row r="62" spans="2:5">
       <c r="B62" s="35"/>
     </row>
-    <row r="63" spans="2:5" ht="29">
+    <row r="63" spans="2:5" ht="30">
       <c r="B63" s="41" t="s">
         <v>528</v>
       </c>
@@ -7864,7 +8148,7 @@
     <row r="70" spans="2:2">
       <c r="B70" s="35"/>
     </row>
-    <row r="71" spans="2:2" ht="29">
+    <row r="71" spans="2:2" ht="30">
       <c r="B71" s="41" t="s">
         <v>531</v>
       </c>
@@ -7936,7 +8220,7 @@
     <row r="87" spans="2:2">
       <c r="B87" s="35"/>
     </row>
-    <row r="88" spans="2:2" ht="29">
+    <row r="88" spans="2:2" ht="30">
       <c r="B88" s="41" t="s">
         <v>543</v>
       </c>
@@ -7966,13 +8250,13 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3D44BBD2-A1D4-40C3-89FB-A46E221B6965}">
   <dimension ref="B2:G204"/>
-  <sheetFormatPr defaultRowHeight="18"/>
+  <sheetFormatPr defaultRowHeight="18.75"/>
   <cols>
     <col min="2" max="2" width="16.5" customWidth="1"/>
-    <col min="3" max="7" width="27.58203125" customWidth="1"/>
+    <col min="3" max="7" width="27.625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:7" ht="29">
+    <row r="2" spans="2:7" ht="30">
       <c r="B2" s="30" t="s">
         <v>9</v>
       </c>
@@ -7982,7 +8266,7 @@
         <v>285</v>
       </c>
     </row>
-    <row r="6" spans="2:7" ht="29">
+    <row r="6" spans="2:7" ht="30">
       <c r="B6" s="30" t="s">
         <v>286</v>
       </c>
@@ -8047,7 +8331,7 @@
         <v>299</v>
       </c>
     </row>
-    <row r="11" spans="2:7" ht="54">
+    <row r="11" spans="2:7" ht="56.25">
       <c r="B11" s="32">
         <v>3</v>
       </c>
@@ -8067,7 +8351,7 @@
         <v>304</v>
       </c>
     </row>
-    <row r="12" spans="2:7" ht="72">
+    <row r="12" spans="2:7" ht="75">
       <c r="B12" s="32">
         <v>4</v>
       </c>
@@ -8087,7 +8371,7 @@
         <v>308</v>
       </c>
     </row>
-    <row r="13" spans="2:7" ht="36">
+    <row r="13" spans="2:7" ht="37.5">
       <c r="B13" s="32">
         <v>5</v>
       </c>
@@ -8107,7 +8391,7 @@
         <v>308</v>
       </c>
     </row>
-    <row r="14" spans="2:7" ht="36">
+    <row r="14" spans="2:7" ht="37.5">
       <c r="B14" s="32">
         <v>6</v>
       </c>
@@ -8127,7 +8411,7 @@
         <v>308</v>
       </c>
     </row>
-    <row r="15" spans="2:7" ht="36">
+    <row r="15" spans="2:7" ht="37.5">
       <c r="B15" s="32">
         <v>7</v>
       </c>
@@ -8147,7 +8431,7 @@
         <v>316</v>
       </c>
     </row>
-    <row r="16" spans="2:7" ht="36">
+    <row r="16" spans="2:7" ht="37.5">
       <c r="B16" s="32">
         <v>8</v>
       </c>
@@ -8167,7 +8451,7 @@
         <v>308</v>
       </c>
     </row>
-    <row r="17" spans="2:7" ht="36">
+    <row r="17" spans="2:7" ht="37.5">
       <c r="B17" s="32">
         <v>9</v>
       </c>
@@ -8207,7 +8491,7 @@
         <v>308</v>
       </c>
     </row>
-    <row r="19" spans="2:7" ht="36">
+    <row r="19" spans="2:7" ht="37.5">
       <c r="B19" s="32">
         <v>11</v>
       </c>
@@ -8447,7 +8731,7 @@
         <v>316</v>
       </c>
     </row>
-    <row r="31" spans="2:7" ht="36">
+    <row r="31" spans="2:7" ht="37.5">
       <c r="B31" s="32">
         <v>23</v>
       </c>
@@ -8467,7 +8751,7 @@
         <v>316</v>
       </c>
     </row>
-    <row r="32" spans="2:7" ht="36">
+    <row r="32" spans="2:7" ht="37.5">
       <c r="B32" s="32">
         <v>24</v>
       </c>
@@ -8487,7 +8771,7 @@
         <v>360</v>
       </c>
     </row>
-    <row r="33" spans="2:7" ht="36">
+    <row r="33" spans="2:7" ht="37.5">
       <c r="B33" s="32">
         <v>25</v>
       </c>
@@ -8507,7 +8791,7 @@
         <v>364</v>
       </c>
     </row>
-    <row r="34" spans="2:7" ht="36">
+    <row r="34" spans="2:7" ht="37.5">
       <c r="B34" s="32">
         <v>26</v>
       </c>
@@ -8527,12 +8811,12 @@
         <v>368</v>
       </c>
     </row>
-    <row r="37" spans="2:7" ht="29">
+    <row r="37" spans="2:7" ht="30">
       <c r="B37" s="30" t="s">
         <v>369</v>
       </c>
     </row>
-    <row r="39" spans="2:7" ht="22">
+    <row r="39" spans="2:7" ht="22.5">
       <c r="B39" s="33" t="s">
         <v>370</v>
       </c>
@@ -8598,7 +8882,7 @@
         <v>380</v>
       </c>
     </row>
-    <row r="59" spans="2:2" ht="22">
+    <row r="59" spans="2:2" ht="22.5">
       <c r="B59" s="33" t="s">
         <v>381</v>
       </c>
@@ -8641,7 +8925,7 @@
         <v>388</v>
       </c>
     </row>
-    <row r="70" spans="2:2" ht="22">
+    <row r="70" spans="2:2" ht="22.5">
       <c r="B70" s="33" t="s">
         <v>389</v>
       </c>
@@ -8707,7 +8991,7 @@
         <v>398</v>
       </c>
     </row>
-    <row r="90" spans="2:2" ht="22">
+    <row r="90" spans="2:2" ht="22.5">
       <c r="B90" s="33" t="s">
         <v>399</v>
       </c>
@@ -8725,7 +9009,7 @@
         <v>401</v>
       </c>
     </row>
-    <row r="96" spans="2:2" ht="22">
+    <row r="96" spans="2:2" ht="22.5">
       <c r="B96" s="33" t="s">
         <v>402</v>
       </c>
@@ -8743,7 +9027,7 @@
         <v>404</v>
       </c>
     </row>
-    <row r="102" spans="2:2" ht="22">
+    <row r="102" spans="2:2" ht="22.5">
       <c r="B102" s="33" t="s">
         <v>405</v>
       </c>
@@ -8761,7 +9045,7 @@
         <v>407</v>
       </c>
     </row>
-    <row r="108" spans="2:2" ht="22">
+    <row r="108" spans="2:2" ht="22.5">
       <c r="B108" s="33" t="s">
         <v>408</v>
       </c>
@@ -8784,7 +9068,7 @@
         <v>411</v>
       </c>
     </row>
-    <row r="115" spans="2:2" ht="22">
+    <row r="115" spans="2:2" ht="22.5">
       <c r="B115" s="33" t="s">
         <v>412</v>
       </c>
@@ -8802,7 +9086,7 @@
         <v>414</v>
       </c>
     </row>
-    <row r="121" spans="2:2" ht="22">
+    <row r="121" spans="2:2" ht="22.5">
       <c r="B121" s="33" t="s">
         <v>415</v>
       </c>
@@ -8820,7 +9104,7 @@
         <v>417</v>
       </c>
     </row>
-    <row r="127" spans="2:2" ht="22">
+    <row r="127" spans="2:2" ht="22.5">
       <c r="B127" s="33" t="s">
         <v>418</v>
       </c>
@@ -8838,7 +9122,7 @@
         <v>420</v>
       </c>
     </row>
-    <row r="133" spans="2:2" ht="22">
+    <row r="133" spans="2:2" ht="22.5">
       <c r="B133" s="33" t="s">
         <v>421</v>
       </c>
@@ -8856,7 +9140,7 @@
         <v>423</v>
       </c>
     </row>
-    <row r="139" spans="2:2" ht="22">
+    <row r="139" spans="2:2" ht="22.5">
       <c r="B139" s="33" t="s">
         <v>424</v>
       </c>
@@ -8874,7 +9158,7 @@
         <v>426</v>
       </c>
     </row>
-    <row r="145" spans="2:2" ht="22">
+    <row r="145" spans="2:2" ht="22.5">
       <c r="B145" s="33" t="s">
         <v>427</v>
       </c>
@@ -8892,7 +9176,7 @@
         <v>429</v>
       </c>
     </row>
-    <row r="151" spans="2:2" ht="22">
+    <row r="151" spans="2:2" ht="22.5">
       <c r="B151" s="33" t="s">
         <v>430</v>
       </c>
@@ -8910,7 +9194,7 @@
         <v>432</v>
       </c>
     </row>
-    <row r="157" spans="2:2" ht="22">
+    <row r="157" spans="2:2" ht="22.5">
       <c r="B157" s="33" t="s">
         <v>433</v>
       </c>
@@ -8981,7 +9265,7 @@
         <v>445</v>
       </c>
     </row>
-    <row r="176" spans="2:2" ht="22">
+    <row r="176" spans="2:2" ht="22.5">
       <c r="B176" s="33" t="s">
         <v>446</v>
       </c>
@@ -8999,7 +9283,7 @@
         <v>448</v>
       </c>
     </row>
-    <row r="182" spans="2:2" ht="22">
+    <row r="182" spans="2:2" ht="22.5">
       <c r="B182" s="33" t="s">
         <v>449</v>
       </c>
@@ -9032,7 +9316,7 @@
         <v>454</v>
       </c>
     </row>
-    <row r="193" spans="2:4" ht="29">
+    <row r="193" spans="2:4" ht="30">
       <c r="B193" s="30" t="s">
         <v>455</v>
       </c>
@@ -9048,7 +9332,7 @@
         <v>456</v>
       </c>
     </row>
-    <row r="196" spans="2:4" ht="36">
+    <row r="196" spans="2:4" ht="37.5">
       <c r="B196" s="32" t="s">
         <v>457</v>
       </c>
@@ -9059,7 +9343,7 @@
         <v>458</v>
       </c>
     </row>
-    <row r="197" spans="2:4" ht="36">
+    <row r="197" spans="2:4" ht="37.5">
       <c r="B197" s="32" t="s">
         <v>459</v>
       </c>
@@ -9070,7 +9354,7 @@
         <v>460</v>
       </c>
     </row>
-    <row r="200" spans="2:4" ht="29">
+    <row r="200" spans="2:4" ht="30">
       <c r="B200" s="30" t="s">
         <v>461</v>
       </c>
@@ -9102,17 +9386,17 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6D8D6D56-B5C7-4754-AB8D-4CB98E7AAD79}">
   <dimension ref="B2:E179"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15.75"/>
   <cols>
     <col min="1" max="1" width="9" style="28"/>
     <col min="2" max="2" width="96.5" style="28" customWidth="1"/>
     <col min="3" max="3" width="24.25" style="28" customWidth="1"/>
     <col min="4" max="4" width="23.5" style="28" customWidth="1"/>
-    <col min="5" max="5" width="26.33203125" style="28" customWidth="1"/>
+    <col min="5" max="5" width="26.375" style="28" customWidth="1"/>
     <col min="6" max="16384" width="9" style="28"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:2" ht="24.5">
+    <row r="2" spans="2:2" ht="24">
       <c r="B2" s="48" t="s">
         <v>465</v>
       </c>
@@ -9122,12 +9406,12 @@
         <v>546</v>
       </c>
     </row>
-    <row r="8" spans="2:2" ht="24.5">
+    <row r="8" spans="2:2" ht="24">
       <c r="B8" s="48" t="s">
         <v>547</v>
       </c>
     </row>
-    <row r="10" spans="2:2" ht="19">
+    <row r="10" spans="2:2" ht="18.75">
       <c r="B10" s="49" t="s">
         <v>548</v>
       </c>
@@ -9237,7 +9521,7 @@
         <v>638</v>
       </c>
     </row>
-    <row r="29" spans="2:5" ht="19">
+    <row r="29" spans="2:5" ht="18.75">
       <c r="B29" s="49" t="s">
         <v>570</v>
       </c>
@@ -9452,7 +9736,7 @@
         <v>641</v>
       </c>
     </row>
-    <row r="92" spans="2:2" ht="19">
+    <row r="92" spans="2:2" ht="18.75">
       <c r="B92" s="49" t="s">
         <v>608</v>
       </c>
@@ -9467,7 +9751,7 @@
         <v>609</v>
       </c>
     </row>
-    <row r="98" spans="2:2" ht="19">
+    <row r="98" spans="2:2" ht="18.75">
       <c r="B98" s="49" t="s">
         <v>610</v>
       </c>
@@ -9550,7 +9834,7 @@
         <v>622</v>
       </c>
     </row>
-    <row r="123" spans="2:2" ht="19">
+    <row r="123" spans="2:2" ht="18.75">
       <c r="B123" s="49" t="s">
         <v>623</v>
       </c>
@@ -9565,7 +9849,7 @@
         <v>647</v>
       </c>
     </row>
-    <row r="131" spans="2:3" ht="24.5">
+    <row r="131" spans="2:3" ht="24">
       <c r="B131" s="48" t="s">
         <v>62</v>
       </c>
@@ -9578,7 +9862,7 @@
         <v>624</v>
       </c>
     </row>
-    <row r="134" spans="2:3" ht="30">
+    <row r="134" spans="2:3" ht="31.5">
       <c r="B134" s="56" t="s">
         <v>625</v>
       </c>
@@ -9586,7 +9870,7 @@
         <v>626</v>
       </c>
     </row>
-    <row r="135" spans="2:3" ht="30">
+    <row r="135" spans="2:3" ht="31.5">
       <c r="B135" s="56" t="s">
         <v>627</v>
       </c>
@@ -9594,7 +9878,7 @@
         <v>628</v>
       </c>
     </row>
-    <row r="136" spans="2:3" ht="30">
+    <row r="136" spans="2:3" ht="31.5">
       <c r="B136" s="56" t="s">
         <v>66</v>
       </c>
@@ -9602,7 +9886,7 @@
         <v>629</v>
       </c>
     </row>
-    <row r="139" spans="2:3" ht="24.5">
+    <row r="139" spans="2:3" ht="24">
       <c r="B139" s="48" t="s">
         <v>461</v>
       </c>
@@ -9661,7 +9945,7 @@
       <c r="D152" s="71"/>
       <c r="E152" s="71"/>
     </row>
-    <row r="154" spans="2:5" ht="24.5">
+    <row r="154" spans="2:5" ht="24">
       <c r="B154" s="58" t="s">
         <v>290</v>
       </c>
@@ -9671,7 +9955,7 @@
         <v>650</v>
       </c>
     </row>
-    <row r="156" spans="2:5" ht="19">
+    <row r="156" spans="2:5" ht="18.75">
       <c r="B156" s="60" t="s">
         <v>651</v>
       </c>
@@ -9722,7 +10006,7 @@
     <row r="166" spans="2:3">
       <c r="B166" s="52"/>
     </row>
-    <row r="167" spans="2:3" ht="19">
+    <row r="167" spans="2:3" ht="18.75">
       <c r="B167" s="60" t="s">
         <v>656</v>
       </c>
@@ -9732,7 +10016,7 @@
         <v>667</v>
       </c>
     </row>
-    <row r="169" spans="2:3" ht="24.5">
+    <row r="169" spans="2:3" ht="24">
       <c r="B169" s="58" t="s">
         <v>657</v>
       </c>
@@ -9745,7 +10029,7 @@
         <v>658</v>
       </c>
     </row>
-    <row r="171" spans="2:3" ht="90.5" thickBot="1">
+    <row r="171" spans="2:3" ht="95.25" thickBot="1">
       <c r="B171" s="66" t="s">
         <v>659</v>
       </c>
@@ -9753,7 +10037,7 @@
         <v>668</v>
       </c>
     </row>
-    <row r="172" spans="2:3" ht="30.5" thickBot="1">
+    <row r="172" spans="2:3" ht="32.25" thickBot="1">
       <c r="B172" s="66" t="s">
         <v>660</v>
       </c>
@@ -9761,7 +10045,7 @@
         <v>669</v>
       </c>
     </row>
-    <row r="173" spans="2:3" ht="45">
+    <row r="173" spans="2:3" ht="47.25">
       <c r="B173" s="66" t="s">
         <v>66</v>
       </c>
@@ -9769,7 +10053,7 @@
         <v>661</v>
       </c>
     </row>
-    <row r="174" spans="2:3" ht="24.5">
+    <row r="174" spans="2:3" ht="24">
       <c r="B174" s="58" t="s">
         <v>662</v>
       </c>
@@ -9795,6 +10079,184 @@
     <row r="179" spans="2:2" ht="19.5">
       <c r="B179" s="70" t="s">
         <v>673</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1152C09E-8861-45D9-9023-348534451E04}">
+  <dimension ref="B1:D29"/>
+  <sheetFormatPr defaultRowHeight="16.5"/>
+  <cols>
+    <col min="1" max="1" width="9" style="72"/>
+    <col min="2" max="2" width="79.25" style="72" customWidth="1"/>
+    <col min="3" max="16384" width="9" style="72"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="2:2">
+      <c r="B1" s="73" t="s">
+        <v>678</v>
+      </c>
+    </row>
+    <row r="2" spans="2:2">
+      <c r="B2" s="73" t="s">
+        <v>679</v>
+      </c>
+    </row>
+    <row r="3" spans="2:2">
+      <c r="B3" s="74" t="s">
+        <v>701</v>
+      </c>
+    </row>
+    <row r="5" spans="2:2">
+      <c r="B5" s="73" t="s">
+        <v>680</v>
+      </c>
+    </row>
+    <row r="6" spans="2:2">
+      <c r="B6" s="73" t="s">
+        <v>681</v>
+      </c>
+    </row>
+    <row r="7" spans="2:2">
+      <c r="B7" s="74" t="s">
+        <v>682</v>
+      </c>
+    </row>
+    <row r="8" spans="2:2" ht="56.25" customHeight="1">
+      <c r="B8" s="72" t="s">
+        <v>683</v>
+      </c>
+    </row>
+    <row r="9" spans="2:2">
+      <c r="B9" s="72" t="s">
+        <v>684</v>
+      </c>
+    </row>
+    <row r="10" spans="2:2" ht="66">
+      <c r="B10" s="74" t="s">
+        <v>702</v>
+      </c>
+    </row>
+    <row r="11" spans="2:2">
+      <c r="B11" s="73" t="s">
+        <v>685</v>
+      </c>
+    </row>
+    <row r="12" spans="2:2" ht="33">
+      <c r="B12" s="74" t="s">
+        <v>686</v>
+      </c>
+    </row>
+    <row r="13" spans="2:2">
+      <c r="B13" s="75"/>
+    </row>
+    <row r="14" spans="2:2">
+      <c r="B14" s="75" t="s">
+        <v>703</v>
+      </c>
+    </row>
+    <row r="15" spans="2:2">
+      <c r="B15" s="76" t="s">
+        <v>704</v>
+      </c>
+    </row>
+    <row r="16" spans="2:2">
+      <c r="B16" s="74"/>
+    </row>
+    <row r="17" spans="2:4">
+      <c r="B17" s="73" t="s">
+        <v>705</v>
+      </c>
+    </row>
+    <row r="18" spans="2:4" ht="33">
+      <c r="B18" s="74" t="s">
+        <v>687</v>
+      </c>
+    </row>
+    <row r="20" spans="2:4">
+      <c r="B20" s="73" t="s">
+        <v>688</v>
+      </c>
+    </row>
+    <row r="21" spans="2:4" ht="49.5">
+      <c r="B21" s="74" t="s">
+        <v>706</v>
+      </c>
+    </row>
+    <row r="23" spans="2:4">
+      <c r="B23" s="73" t="s">
+        <v>689</v>
+      </c>
+    </row>
+    <row r="24" spans="2:4">
+      <c r="B24" s="77" t="s">
+        <v>690</v>
+      </c>
+      <c r="C24" s="77" t="s">
+        <v>63</v>
+      </c>
+      <c r="D24" s="78" t="s">
+        <v>691</v>
+      </c>
+    </row>
+    <row r="25" spans="2:4" ht="215.25" thickBot="1">
+      <c r="B25" s="79" t="s">
+        <v>692</v>
+      </c>
+      <c r="C25" s="80" t="s">
+        <v>693</v>
+      </c>
+      <c r="D25" s="81" t="s">
+        <v>707</v>
+      </c>
+    </row>
+    <row r="26" spans="2:4" ht="132.75" thickBot="1">
+      <c r="B26" s="79" t="s">
+        <v>694</v>
+      </c>
+      <c r="C26" s="80" t="s">
+        <v>659</v>
+      </c>
+      <c r="D26" s="81" t="s">
+        <v>695</v>
+      </c>
+    </row>
+    <row r="27" spans="2:4" ht="66.75" thickBot="1">
+      <c r="B27" s="79" t="s">
+        <v>696</v>
+      </c>
+      <c r="C27" s="80" t="s">
+        <v>660</v>
+      </c>
+      <c r="D27" s="81" t="s">
+        <v>697</v>
+      </c>
+    </row>
+    <row r="28" spans="2:4" ht="132.75" thickBot="1">
+      <c r="B28" s="79" t="s">
+        <v>698</v>
+      </c>
+      <c r="C28" s="80" t="s">
+        <v>699</v>
+      </c>
+      <c r="D28" s="81" t="s">
+        <v>708</v>
+      </c>
+    </row>
+    <row r="29" spans="2:4" ht="198">
+      <c r="B29" s="79" t="s">
+        <v>700</v>
+      </c>
+      <c r="C29" s="80" t="s">
+        <v>66</v>
+      </c>
+      <c r="D29" s="74" t="s">
+        <v>709</v>
       </c>
     </row>
   </sheetData>

</xml_diff>